<commit_message>
codex - initialize to full hp mp.
</commit_message>
<xml_diff>
--- a/jyx2/Assets/Mods/jshyl/Configs/人物.xlsx
+++ b/jyx2/Assets/Mods/jshyl/Configs/人物.xlsx
@@ -1129,7 +1129,7 @@
         <v>0</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>3</v>
+        <v>100</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
@@ -1145,16 +1145,16 @@
         <v>0</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>0</v>
+        <v>999999</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>38</v>
+        <v>9999</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>38</v>
+        <v>999</v>
       </c>
       <c r="K5" s="2" t="n">
         <v>0</v>
@@ -1166,7 +1166,7 @@
         <v>100</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>0</v>
+        <v>999</v>
       </c>
       <c r="O5" s="2" t="n">
         <v>-1</v>
@@ -1175,77 +1175,77 @@
         <v>-1</v>
       </c>
       <c r="Q5" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R5" s="2" t="n">
-        <v>26</v>
+        <v>9999</v>
       </c>
       <c r="S5" s="2" t="n">
-        <v>26</v>
+        <v>999</v>
       </c>
       <c r="T5" s="2" t="n">
-        <v>27</v>
+        <v>999</v>
       </c>
       <c r="U5" s="2" t="n">
-        <v>27</v>
+        <v>999</v>
       </c>
       <c r="V5" s="2" t="n">
-        <v>27</v>
+        <v>999</v>
       </c>
       <c r="W5" s="2" t="n">
-        <v>30</v>
+        <v>999</v>
       </c>
       <c r="X5" s="2" t="n">
-        <v>30</v>
+        <v>999</v>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>23</v>
+        <v>999</v>
       </c>
       <c r="Z5" s="2" t="n">
-        <v>25</v>
+        <v>999</v>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>30</v>
+        <v>999</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>28</v>
+        <v>999</v>
       </c>
       <c r="AC5" s="2" t="n">
-        <v>26</v>
+        <v>999</v>
       </c>
       <c r="AD5" s="2" t="n">
-        <v>24</v>
+        <v>999</v>
       </c>
       <c r="AE5" s="2" t="n">
-        <v>25</v>
+        <v>999</v>
       </c>
       <c r="AF5" s="2" t="n">
-        <v>0</v>
+        <v>999</v>
       </c>
       <c r="AG5" s="2" t="n">
-        <v>50</v>
+        <v>999</v>
       </c>
       <c r="AH5" s="2" t="n">
-        <v>0</v>
+        <v>999</v>
       </c>
       <c r="AI5" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>0</v>
+        <v>999</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>39</v>
+        <v>100</v>
       </c>
       <c r="AL5" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="AM5" s="2" t="n">
-        <v>0</v>
+        <v>999</v>
       </c>
       <c r="AN5" s="5" t="inlineStr">
         <is>
-          <t>1,0</t>
+          <t>1,900|25,900|30,900|57,900|58,900|61,900|87,900|92,900|29,900|205,900</t>
         </is>
       </c>
       <c r="AO5" s="5" t="inlineStr">
@@ -43474,1836 +43474,1836 @@
       </c>
     </row>
     <row r="326">
-      <c r="A326" t="n">
+      <c r="A326" s="0" t="n">
         <v>321</v>
       </c>
-      <c r="B326" t="n">
+      <c r="B326" s="0" t="n">
         <v>65</v>
       </c>
-      <c r="C326" t="n">
+      <c r="C326" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="D326" t="inlineStr">
+      <c r="D326" s="0" t="inlineStr">
         <is>
           <t>觉远</t>
         </is>
       </c>
-      <c r="E326" t="inlineStr">
+      <c r="E326" s="0" t="inlineStr">
         <is>
           <t>少林高僧</t>
         </is>
       </c>
-      <c r="F326" t="n">
-        <v>0</v>
-      </c>
-      <c r="G326" t="n">
+      <c r="F326" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G326" s="0" t="n">
         <v>18</v>
       </c>
-      <c r="H326" t="n">
+      <c r="H326" s="0" t="n">
         <v>12000</v>
       </c>
-      <c r="I326" t="n">
+      <c r="I326" s="0" t="n">
         <v>260</v>
       </c>
-      <c r="J326" t="n">
+      <c r="J326" s="0" t="n">
         <v>260</v>
       </c>
-      <c r="K326" t="n">
-        <v>0</v>
-      </c>
-      <c r="L326" t="n">
-        <v>0</v>
-      </c>
-      <c r="M326" t="n">
+      <c r="K326" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="L326" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M326" s="0" t="n">
         <v>450</v>
       </c>
-      <c r="N326" t="n">
-        <v>0</v>
-      </c>
-      <c r="O326" t="n">
-        <v>-1</v>
-      </c>
-      <c r="P326" t="n">
-        <v>-1</v>
-      </c>
-      <c r="Q326" t="n">
+      <c r="N326" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O326" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="P326" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="Q326" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="R326" t="n">
+      <c r="R326" s="0" t="n">
         <v>120</v>
       </c>
-      <c r="S326" t="n">
+      <c r="S326" s="0" t="n">
         <v>120</v>
       </c>
-      <c r="T326" t="n">
+      <c r="T326" s="0" t="n">
         <v>72</v>
       </c>
-      <c r="U326" t="n">
+      <c r="U326" s="0" t="n">
         <v>50</v>
       </c>
-      <c r="V326" t="n">
+      <c r="V326" s="0" t="n">
         <v>82</v>
       </c>
-      <c r="W326" t="n">
-        <v>0</v>
-      </c>
-      <c r="X326" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y326" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z326" t="n">
+      <c r="W326" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="X326" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y326" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z326" s="0" t="n">
         <v>60</v>
       </c>
-      <c r="AA326" t="n">
+      <c r="AA326" s="0" t="n">
         <v>20</v>
       </c>
-      <c r="AB326" t="n">
+      <c r="AB326" s="0" t="n">
         <v>30</v>
       </c>
-      <c r="AC326" t="n">
-        <v>10</v>
-      </c>
-      <c r="AD326" t="n">
+      <c r="AC326" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AD326" s="0" t="n">
         <v>50</v>
       </c>
-      <c r="AE326" t="n">
-        <v>10</v>
-      </c>
-      <c r="AF326" t="n">
-        <v>10</v>
-      </c>
-      <c r="AG326" t="n">
+      <c r="AE326" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AF326" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AG326" s="0" t="n">
         <v>60</v>
       </c>
-      <c r="AH326" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI326" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ326" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK326" t="n">
+      <c r="AH326" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI326" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ326" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK326" s="0" t="n">
         <v>70</v>
       </c>
-      <c r="AL326" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AM326" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN326" t="inlineStr">
+      <c r="AL326" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AM326" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN326" s="0" t="inlineStr">
         <is>
           <t>1,350</t>
         </is>
       </c>
-      <c r="AO326" t="n">
+      <c r="AO326" s="0" t="n">
         <v>-1</v>
       </c>
     </row>
     <row r="327">
-      <c r="A327" t="n">
+      <c r="A327" s="0" t="n">
         <v>322</v>
       </c>
-      <c r="B327" t="n">
+      <c r="B327" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="C327" t="n">
+      <c r="C327" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="D327" t="inlineStr">
+      <c r="D327" s="0" t="inlineStr">
         <is>
           <t>何足道</t>
         </is>
       </c>
-      <c r="E327" t="inlineStr">
+      <c r="E327" s="0" t="inlineStr">
         <is>
           <t>昆仑三圣</t>
         </is>
       </c>
-      <c r="F327" t="n">
-        <v>0</v>
-      </c>
-      <c r="G327" t="n">
+      <c r="F327" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G327" s="0" t="n">
         <v>20</v>
       </c>
-      <c r="H327" t="n">
+      <c r="H327" s="0" t="n">
         <v>16250</v>
       </c>
-      <c r="I327" t="n">
+      <c r="I327" s="0" t="n">
         <v>300</v>
       </c>
-      <c r="J327" t="n">
+      <c r="J327" s="0" t="n">
         <v>300</v>
       </c>
-      <c r="K327" t="n">
-        <v>0</v>
-      </c>
-      <c r="L327" t="n">
-        <v>0</v>
-      </c>
-      <c r="M327" t="n">
+      <c r="K327" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="L327" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M327" s="0" t="n">
         <v>500</v>
       </c>
-      <c r="N327" t="n">
-        <v>0</v>
-      </c>
-      <c r="O327" t="n">
-        <v>-1</v>
-      </c>
-      <c r="P327" t="n">
-        <v>-1</v>
-      </c>
-      <c r="Q327" t="n">
+      <c r="N327" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O327" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="P327" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="Q327" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="R327" t="n">
+      <c r="R327" s="0" t="n">
         <v>110</v>
       </c>
-      <c r="S327" t="n">
+      <c r="S327" s="0" t="n">
         <v>110</v>
       </c>
-      <c r="T327" t="n">
+      <c r="T327" s="0" t="n">
         <v>78</v>
       </c>
-      <c r="U327" t="n">
+      <c r="U327" s="0" t="n">
         <v>68</v>
       </c>
-      <c r="V327" t="n">
+      <c r="V327" s="0" t="n">
         <v>78</v>
       </c>
-      <c r="W327" t="n">
-        <v>0</v>
-      </c>
-      <c r="X327" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y327" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z327" t="n">
+      <c r="W327" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="X327" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y327" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z327" s="0" t="n">
         <v>20</v>
       </c>
-      <c r="AA327" t="n">
-        <v>10</v>
-      </c>
-      <c r="AB327" t="n">
+      <c r="AA327" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AB327" s="0" t="n">
         <v>20</v>
       </c>
-      <c r="AC327" t="n">
+      <c r="AC327" s="0" t="n">
         <v>12</v>
       </c>
-      <c r="AD327" t="n">
+      <c r="AD327" s="0" t="n">
         <v>82</v>
       </c>
-      <c r="AE327" t="n">
-        <v>10</v>
-      </c>
-      <c r="AF327" t="n">
+      <c r="AE327" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AF327" s="0" t="n">
         <v>70</v>
       </c>
-      <c r="AG327" t="n">
+      <c r="AG327" s="0" t="n">
         <v>55</v>
       </c>
-      <c r="AH327" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI327" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ327" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK327" t="n">
+      <c r="AH327" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI327" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ327" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK327" s="0" t="n">
         <v>78</v>
       </c>
-      <c r="AL327" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AM327" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN327" t="inlineStr">
+      <c r="AL327" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AM327" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN327" s="0" t="inlineStr">
         <is>
           <t>1,350</t>
         </is>
       </c>
-      <c r="AO327" t="n">
+      <c r="AO327" s="0" t="n">
         <v>-1</v>
       </c>
     </row>
     <row r="328">
-      <c r="A328" t="n">
+      <c r="A328" s="0" t="n">
         <v>323</v>
       </c>
-      <c r="B328" t="n">
+      <c r="B328" s="0" t="n">
         <v>100</v>
       </c>
-      <c r="C328" t="n">
+      <c r="C328" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="D328" t="inlineStr">
+      <c r="D328" s="0" t="inlineStr">
         <is>
           <t>白猿</t>
         </is>
       </c>
-      <c r="E328" t="inlineStr">
+      <c r="E328" s="0" t="inlineStr">
         <is>
           <t>白公公</t>
         </is>
       </c>
-      <c r="F328" t="n">
-        <v>0</v>
-      </c>
-      <c r="G328" t="n">
+      <c r="F328" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G328" s="0" t="n">
         <v>16</v>
       </c>
-      <c r="H328" t="n">
+      <c r="H328" s="0" t="n">
         <v>9250</v>
       </c>
-      <c r="I328" t="n">
+      <c r="I328" s="0" t="n">
         <v>340</v>
       </c>
-      <c r="J328" t="n">
+      <c r="J328" s="0" t="n">
         <v>340</v>
       </c>
-      <c r="K328" t="n">
-        <v>0</v>
-      </c>
-      <c r="L328" t="n">
-        <v>0</v>
-      </c>
-      <c r="M328" t="n">
-        <v>0</v>
-      </c>
-      <c r="N328" t="n">
-        <v>0</v>
-      </c>
-      <c r="O328" t="n">
-        <v>-1</v>
-      </c>
-      <c r="P328" t="n">
-        <v>-1</v>
-      </c>
-      <c r="Q328" t="n">
+      <c r="K328" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="L328" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M328" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="N328" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O328" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="P328" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="Q328" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="R328" t="n">
+      <c r="R328" s="0" t="n">
         <v>20</v>
       </c>
-      <c r="S328" t="n">
+      <c r="S328" s="0" t="n">
         <v>20</v>
       </c>
-      <c r="T328" t="n">
+      <c r="T328" s="0" t="n">
         <v>85</v>
       </c>
-      <c r="U328" t="n">
+      <c r="U328" s="0" t="n">
         <v>78</v>
       </c>
-      <c r="V328" t="n">
+      <c r="V328" s="0" t="n">
         <v>65</v>
       </c>
-      <c r="W328" t="n">
-        <v>0</v>
-      </c>
-      <c r="X328" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y328" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z328" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA328" t="n">
-        <v>10</v>
-      </c>
-      <c r="AB328" t="n">
-        <v>10</v>
-      </c>
-      <c r="AC328" t="n">
+      <c r="W328" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="X328" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y328" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z328" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA328" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AB328" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AC328" s="0" t="n">
         <v>80</v>
       </c>
-      <c r="AD328" t="n">
-        <v>10</v>
-      </c>
-      <c r="AE328" t="n">
-        <v>10</v>
-      </c>
-      <c r="AF328" t="n">
-        <v>10</v>
-      </c>
-      <c r="AG328" t="n">
+      <c r="AD328" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AE328" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AF328" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AG328" s="0" t="n">
         <v>45</v>
       </c>
-      <c r="AH328" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI328" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ328" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK328" t="n">
+      <c r="AH328" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI328" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ328" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK328" s="0" t="n">
         <v>45</v>
       </c>
-      <c r="AL328" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AM328" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN328" t="inlineStr">
+      <c r="AL328" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AM328" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN328" s="0" t="inlineStr">
         <is>
           <t>1,250</t>
         </is>
       </c>
-      <c r="AO328" t="n">
+      <c r="AO328" s="0" t="n">
         <v>-1</v>
       </c>
     </row>
     <row r="329">
-      <c r="A329" t="n">
+      <c r="A329" s="0" t="n">
         <v>324</v>
       </c>
-      <c r="B329" t="n">
+      <c r="B329" s="0" t="n">
         <v>65</v>
       </c>
-      <c r="C329" t="n">
+      <c r="C329" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="D329" t="inlineStr">
+      <c r="D329" s="0" t="inlineStr">
         <is>
           <t>无相</t>
         </is>
       </c>
-      <c r="E329" t="inlineStr">
+      <c r="E329" s="0" t="inlineStr">
         <is>
           <t>西域僧</t>
         </is>
       </c>
-      <c r="F329" t="n">
-        <v>0</v>
-      </c>
-      <c r="G329" t="n">
+      <c r="F329" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G329" s="0" t="n">
         <v>12</v>
       </c>
-      <c r="H329" t="n">
+      <c r="H329" s="0" t="n">
         <v>3850</v>
       </c>
-      <c r="I329" t="n">
+      <c r="I329" s="0" t="n">
         <v>210</v>
       </c>
-      <c r="J329" t="n">
+      <c r="J329" s="0" t="n">
         <v>210</v>
       </c>
-      <c r="K329" t="n">
-        <v>0</v>
-      </c>
-      <c r="L329" t="n">
-        <v>0</v>
-      </c>
-      <c r="M329" t="n">
+      <c r="K329" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="L329" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M329" s="0" t="n">
         <v>320</v>
       </c>
-      <c r="N329" t="n">
-        <v>0</v>
-      </c>
-      <c r="O329" t="n">
-        <v>-1</v>
-      </c>
-      <c r="P329" t="n">
-        <v>-1</v>
-      </c>
-      <c r="Q329" t="n">
+      <c r="N329" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O329" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="P329" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="Q329" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="R329" t="n">
+      <c r="R329" s="0" t="n">
         <v>70</v>
       </c>
-      <c r="S329" t="n">
+      <c r="S329" s="0" t="n">
         <v>70</v>
       </c>
-      <c r="T329" t="n">
+      <c r="T329" s="0" t="n">
         <v>62</v>
       </c>
-      <c r="U329" t="n">
+      <c r="U329" s="0" t="n">
         <v>40</v>
       </c>
-      <c r="V329" t="n">
+      <c r="V329" s="0" t="n">
         <v>65</v>
       </c>
-      <c r="W329" t="n">
-        <v>0</v>
-      </c>
-      <c r="X329" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y329" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z329" t="n">
+      <c r="W329" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="X329" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y329" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z329" s="0" t="n">
         <v>50</v>
       </c>
-      <c r="AA329" t="n">
-        <v>10</v>
-      </c>
-      <c r="AB329" t="n">
+      <c r="AA329" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AB329" s="0" t="n">
         <v>20</v>
       </c>
-      <c r="AC329" t="n">
-        <v>10</v>
-      </c>
-      <c r="AD329" t="n">
+      <c r="AC329" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AD329" s="0" t="n">
         <v>30</v>
       </c>
-      <c r="AE329" t="n">
-        <v>10</v>
-      </c>
-      <c r="AF329" t="n">
-        <v>10</v>
-      </c>
-      <c r="AG329" t="n">
+      <c r="AE329" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AF329" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AG329" s="0" t="n">
         <v>45</v>
       </c>
-      <c r="AH329" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI329" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ329" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK329" t="n">
+      <c r="AH329" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI329" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ329" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK329" s="0" t="n">
         <v>55</v>
       </c>
-      <c r="AL329" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AM329" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN329" t="inlineStr">
+      <c r="AL329" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AM329" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN329" s="0" t="inlineStr">
         <is>
           <t>1,250</t>
         </is>
       </c>
-      <c r="AO329" t="n">
+      <c r="AO329" s="0" t="n">
         <v>-1</v>
       </c>
     </row>
     <row r="330">
-      <c r="A330" t="n">
+      <c r="A330" s="0" t="n">
         <v>325</v>
       </c>
-      <c r="B330" t="n">
+      <c r="B330" s="0" t="n">
         <v>64</v>
       </c>
-      <c r="C330" t="n">
+      <c r="C330" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="D330" t="inlineStr">
+      <c r="D330" s="0" t="inlineStr">
         <is>
           <t>无色</t>
         </is>
       </c>
-      <c r="E330" t="inlineStr">
+      <c r="E330" s="0" t="inlineStr">
         <is>
           <t>西域僧</t>
         </is>
       </c>
-      <c r="F330" t="n">
-        <v>0</v>
-      </c>
-      <c r="G330" t="n">
+      <c r="F330" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G330" s="0" t="n">
         <v>12</v>
       </c>
-      <c r="H330" t="n">
+      <c r="H330" s="0" t="n">
         <v>3850</v>
       </c>
-      <c r="I330" t="n">
+      <c r="I330" s="0" t="n">
         <v>210</v>
       </c>
-      <c r="J330" t="n">
+      <c r="J330" s="0" t="n">
         <v>210</v>
       </c>
-      <c r="K330" t="n">
-        <v>0</v>
-      </c>
-      <c r="L330" t="n">
-        <v>0</v>
-      </c>
-      <c r="M330" t="n">
+      <c r="K330" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="L330" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M330" s="0" t="n">
         <v>320</v>
       </c>
-      <c r="N330" t="n">
-        <v>0</v>
-      </c>
-      <c r="O330" t="n">
-        <v>-1</v>
-      </c>
-      <c r="P330" t="n">
-        <v>-1</v>
-      </c>
-      <c r="Q330" t="n">
+      <c r="N330" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O330" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="P330" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="Q330" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="R330" t="n">
+      <c r="R330" s="0" t="n">
         <v>70</v>
       </c>
-      <c r="S330" t="n">
+      <c r="S330" s="0" t="n">
         <v>70</v>
       </c>
-      <c r="T330" t="n">
+      <c r="T330" s="0" t="n">
         <v>62</v>
       </c>
-      <c r="U330" t="n">
+      <c r="U330" s="0" t="n">
         <v>40</v>
       </c>
-      <c r="V330" t="n">
+      <c r="V330" s="0" t="n">
         <v>65</v>
       </c>
-      <c r="W330" t="n">
-        <v>0</v>
-      </c>
-      <c r="X330" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y330" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z330" t="n">
+      <c r="W330" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="X330" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y330" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z330" s="0" t="n">
         <v>50</v>
       </c>
-      <c r="AA330" t="n">
-        <v>10</v>
-      </c>
-      <c r="AB330" t="n">
+      <c r="AA330" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AB330" s="0" t="n">
         <v>20</v>
       </c>
-      <c r="AC330" t="n">
-        <v>10</v>
-      </c>
-      <c r="AD330" t="n">
+      <c r="AC330" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AD330" s="0" t="n">
         <v>30</v>
       </c>
-      <c r="AE330" t="n">
-        <v>10</v>
-      </c>
-      <c r="AF330" t="n">
-        <v>10</v>
-      </c>
-      <c r="AG330" t="n">
+      <c r="AE330" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AF330" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AG330" s="0" t="n">
         <v>45</v>
       </c>
-      <c r="AH330" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI330" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ330" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK330" t="n">
+      <c r="AH330" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI330" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ330" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK330" s="0" t="n">
         <v>55</v>
       </c>
-      <c r="AL330" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AM330" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN330" t="inlineStr">
+      <c r="AL330" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AM330" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN330" s="0" t="inlineStr">
         <is>
           <t>1,250</t>
         </is>
       </c>
-      <c r="AO330" t="n">
+      <c r="AO330" s="0" t="n">
         <v>-1</v>
       </c>
     </row>
     <row r="331">
-      <c r="A331" t="n">
+      <c r="A331" s="0" t="n">
         <v>326</v>
       </c>
-      <c r="B331" t="n">
+      <c r="B331" s="0" t="n">
         <v>71</v>
       </c>
-      <c r="C331" t="n">
+      <c r="C331" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="D331" t="inlineStr">
+      <c r="D331" s="0" t="inlineStr">
         <is>
           <t>尹克西</t>
         </is>
       </c>
-      <c r="E331" t="inlineStr">
+      <c r="E331" s="0" t="inlineStr">
         <is>
           <t>西域高手</t>
         </is>
       </c>
-      <c r="F331" t="n">
-        <v>0</v>
-      </c>
-      <c r="G331" t="n">
+      <c r="F331" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G331" s="0" t="n">
         <v>14</v>
       </c>
-      <c r="H331" t="n">
+      <c r="H331" s="0" t="n">
         <v>6350</v>
       </c>
-      <c r="I331" t="n">
+      <c r="I331" s="0" t="n">
         <v>230</v>
       </c>
-      <c r="J331" t="n">
+      <c r="J331" s="0" t="n">
         <v>230</v>
       </c>
-      <c r="K331" t="n">
-        <v>0</v>
-      </c>
-      <c r="L331" t="n">
-        <v>0</v>
-      </c>
-      <c r="M331" t="n">
+      <c r="K331" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="L331" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M331" s="0" t="n">
         <v>360</v>
       </c>
-      <c r="N331" t="n">
-        <v>0</v>
-      </c>
-      <c r="O331" t="n">
-        <v>-1</v>
-      </c>
-      <c r="P331" t="n">
-        <v>-1</v>
-      </c>
-      <c r="Q331" t="n">
+      <c r="N331" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O331" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="P331" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="Q331" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="R331" t="n">
+      <c r="R331" s="0" t="n">
         <v>75</v>
       </c>
-      <c r="S331" t="n">
+      <c r="S331" s="0" t="n">
         <v>75</v>
       </c>
-      <c r="T331" t="n">
+      <c r="T331" s="0" t="n">
         <v>68</v>
       </c>
-      <c r="U331" t="n">
+      <c r="U331" s="0" t="n">
         <v>42</v>
       </c>
-      <c r="V331" t="n">
+      <c r="V331" s="0" t="n">
         <v>70</v>
       </c>
-      <c r="W331" t="n">
-        <v>0</v>
-      </c>
-      <c r="X331" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y331" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z331" t="n">
+      <c r="W331" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="X331" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y331" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z331" s="0" t="n">
         <v>30</v>
       </c>
-      <c r="AA331" t="n">
-        <v>10</v>
-      </c>
-      <c r="AB331" t="n">
+      <c r="AA331" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AB331" s="0" t="n">
         <v>15</v>
       </c>
-      <c r="AC331" t="n">
-        <v>10</v>
-      </c>
-      <c r="AD331" t="n">
+      <c r="AC331" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AD331" s="0" t="n">
         <v>45</v>
       </c>
-      <c r="AE331" t="n">
-        <v>10</v>
-      </c>
-      <c r="AF331" t="n">
+      <c r="AE331" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AF331" s="0" t="n">
         <v>30</v>
       </c>
-      <c r="AG331" t="n">
+      <c r="AG331" s="0" t="n">
         <v>48</v>
       </c>
-      <c r="AH331" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI331" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ331" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK331" t="n">
+      <c r="AH331" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI331" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ331" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK331" s="0" t="n">
         <v>60</v>
       </c>
-      <c r="AL331" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AM331" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN331" t="inlineStr">
+      <c r="AL331" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AM331" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN331" s="0" t="inlineStr">
         <is>
           <t>1,300</t>
         </is>
       </c>
-      <c r="AO331" t="n">
+      <c r="AO331" s="0" t="n">
         <v>-1</v>
       </c>
     </row>
     <row r="332">
-      <c r="A332" t="n">
+      <c r="A332" s="0" t="n">
         <v>327</v>
       </c>
-      <c r="B332" t="n">
+      <c r="B332" s="0" t="n">
         <v>26</v>
       </c>
-      <c r="C332" t="n">
+      <c r="C332" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="D332" t="inlineStr">
+      <c r="D332" s="0" t="inlineStr">
         <is>
           <t>潇湘子</t>
         </is>
       </c>
-      <c r="E332" t="inlineStr">
+      <c r="E332" s="0" t="inlineStr">
         <is>
           <t>湘西高手</t>
         </is>
       </c>
-      <c r="F332" t="n">
-        <v>0</v>
-      </c>
-      <c r="G332" t="n">
+      <c r="F332" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G332" s="0" t="n">
         <v>14</v>
       </c>
-      <c r="H332" t="n">
+      <c r="H332" s="0" t="n">
         <v>6350</v>
       </c>
-      <c r="I332" t="n">
+      <c r="I332" s="0" t="n">
         <v>230</v>
       </c>
-      <c r="J332" t="n">
+      <c r="J332" s="0" t="n">
         <v>230</v>
       </c>
-      <c r="K332" t="n">
-        <v>0</v>
-      </c>
-      <c r="L332" t="n">
-        <v>0</v>
-      </c>
-      <c r="M332" t="n">
+      <c r="K332" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="L332" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M332" s="0" t="n">
         <v>360</v>
       </c>
-      <c r="N332" t="n">
-        <v>0</v>
-      </c>
-      <c r="O332" t="n">
-        <v>-1</v>
-      </c>
-      <c r="P332" t="n">
-        <v>-1</v>
-      </c>
-      <c r="Q332" t="n">
+      <c r="N332" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O332" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="P332" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="Q332" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="R332" t="n">
+      <c r="R332" s="0" t="n">
         <v>75</v>
       </c>
-      <c r="S332" t="n">
+      <c r="S332" s="0" t="n">
         <v>75</v>
       </c>
-      <c r="T332" t="n">
+      <c r="T332" s="0" t="n">
         <v>65</v>
       </c>
-      <c r="U332" t="n">
+      <c r="U332" s="0" t="n">
         <v>55</v>
       </c>
-      <c r="V332" t="n">
+      <c r="V332" s="0" t="n">
         <v>66</v>
       </c>
-      <c r="W332" t="n">
-        <v>0</v>
-      </c>
-      <c r="X332" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y332" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z332" t="n">
+      <c r="W332" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="X332" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y332" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z332" s="0" t="n">
         <v>40</v>
       </c>
-      <c r="AA332" t="n">
+      <c r="AA332" s="0" t="n">
         <v>25</v>
       </c>
-      <c r="AB332" t="n">
+      <c r="AB332" s="0" t="n">
         <v>25</v>
       </c>
-      <c r="AC332" t="n">
-        <v>10</v>
-      </c>
-      <c r="AD332" t="n">
+      <c r="AC332" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AD332" s="0" t="n">
         <v>55</v>
       </c>
-      <c r="AE332" t="n">
-        <v>10</v>
-      </c>
-      <c r="AF332" t="n">
+      <c r="AE332" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AF332" s="0" t="n">
         <v>30</v>
       </c>
-      <c r="AG332" t="n">
+      <c r="AG332" s="0" t="n">
         <v>40</v>
       </c>
-      <c r="AH332" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI332" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ332" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK332" t="n">
+      <c r="AH332" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI332" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ332" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK332" s="0" t="n">
         <v>62</v>
       </c>
-      <c r="AL332" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AM332" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN332" t="inlineStr">
+      <c r="AL332" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AM332" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN332" s="0" t="inlineStr">
         <is>
           <t>1,300</t>
         </is>
       </c>
-      <c r="AO332" t="n">
+      <c r="AO332" s="0" t="n">
         <v>-1</v>
       </c>
     </row>
     <row r="333">
-      <c r="A333" t="n">
+      <c r="A333" s="0" t="n">
         <v>328</v>
       </c>
-      <c r="B333" t="n">
+      <c r="B333" s="0" t="n">
         <v>71</v>
       </c>
-      <c r="C333" t="n">
+      <c r="C333" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="D333" t="inlineStr">
+      <c r="D333" s="0" t="inlineStr">
         <is>
           <t>西域三僧甲</t>
         </is>
       </c>
-      <c r="E333" t="inlineStr">
+      <c r="E333" s="0" t="inlineStr">
         <is>
           <t>西域三僧</t>
         </is>
       </c>
-      <c r="F333" t="n">
-        <v>0</v>
-      </c>
-      <c r="G333" t="n">
+      <c r="F333" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G333" s="0" t="n">
         <v>11</v>
       </c>
-      <c r="H333" t="n">
+      <c r="H333" s="0" t="n">
         <v>3050</v>
       </c>
-      <c r="I333" t="n">
+      <c r="I333" s="0" t="n">
         <v>190</v>
       </c>
-      <c r="J333" t="n">
+      <c r="J333" s="0" t="n">
         <v>190</v>
       </c>
-      <c r="K333" t="n">
-        <v>0</v>
-      </c>
-      <c r="L333" t="n">
-        <v>0</v>
-      </c>
-      <c r="M333" t="n">
+      <c r="K333" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="L333" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M333" s="0" t="n">
         <v>300</v>
       </c>
-      <c r="N333" t="n">
-        <v>0</v>
-      </c>
-      <c r="O333" t="n">
-        <v>-1</v>
-      </c>
-      <c r="P333" t="n">
-        <v>-1</v>
-      </c>
-      <c r="Q333" t="n">
+      <c r="N333" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O333" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="P333" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="Q333" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="R333" t="n">
+      <c r="R333" s="0" t="n">
         <v>65</v>
       </c>
-      <c r="S333" t="n">
+      <c r="S333" s="0" t="n">
         <v>65</v>
       </c>
-      <c r="T333" t="n">
+      <c r="T333" s="0" t="n">
         <v>58</v>
       </c>
-      <c r="U333" t="n">
+      <c r="U333" s="0" t="n">
         <v>36</v>
       </c>
-      <c r="V333" t="n">
+      <c r="V333" s="0" t="n">
         <v>60</v>
       </c>
-      <c r="W333" t="n">
-        <v>0</v>
-      </c>
-      <c r="X333" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y333" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z333" t="n">
+      <c r="W333" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="X333" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y333" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z333" s="0" t="n">
         <v>45</v>
       </c>
-      <c r="AA333" t="n">
-        <v>10</v>
-      </c>
-      <c r="AB333" t="n">
+      <c r="AA333" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AB333" s="0" t="n">
         <v>15</v>
       </c>
-      <c r="AC333" t="n">
-        <v>10</v>
-      </c>
-      <c r="AD333" t="n">
+      <c r="AC333" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AD333" s="0" t="n">
         <v>25</v>
       </c>
-      <c r="AE333" t="n">
-        <v>10</v>
-      </c>
-      <c r="AF333" t="n">
-        <v>10</v>
-      </c>
-      <c r="AG333" t="n">
+      <c r="AE333" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AF333" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AG333" s="0" t="n">
         <v>42</v>
       </c>
-      <c r="AH333" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI333" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ333" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK333" t="n">
+      <c r="AH333" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI333" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ333" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK333" s="0" t="n">
         <v>50</v>
       </c>
-      <c r="AL333" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AM333" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN333" t="inlineStr">
+      <c r="AL333" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AM333" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN333" s="0" t="inlineStr">
         <is>
           <t>1,220</t>
         </is>
       </c>
-      <c r="AO333" t="n">
+      <c r="AO333" s="0" t="n">
         <v>-1</v>
       </c>
     </row>
     <row r="334">
-      <c r="A334" t="n">
+      <c r="A334" s="0" t="n">
         <v>329</v>
       </c>
-      <c r="B334" t="n">
+      <c r="B334" s="0" t="n">
         <v>71</v>
       </c>
-      <c r="C334" t="n">
+      <c r="C334" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="D334" t="inlineStr">
+      <c r="D334" s="0" t="inlineStr">
         <is>
           <t>西域三僧乙</t>
         </is>
       </c>
-      <c r="E334" t="inlineStr">
+      <c r="E334" s="0" t="inlineStr">
         <is>
           <t>西域三僧</t>
         </is>
       </c>
-      <c r="F334" t="n">
-        <v>0</v>
-      </c>
-      <c r="G334" t="n">
+      <c r="F334" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G334" s="0" t="n">
         <v>11</v>
       </c>
-      <c r="H334" t="n">
+      <c r="H334" s="0" t="n">
         <v>3050</v>
       </c>
-      <c r="I334" t="n">
+      <c r="I334" s="0" t="n">
         <v>190</v>
       </c>
-      <c r="J334" t="n">
+      <c r="J334" s="0" t="n">
         <v>190</v>
       </c>
-      <c r="K334" t="n">
-        <v>0</v>
-      </c>
-      <c r="L334" t="n">
-        <v>0</v>
-      </c>
-      <c r="M334" t="n">
+      <c r="K334" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="L334" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M334" s="0" t="n">
         <v>300</v>
       </c>
-      <c r="N334" t="n">
-        <v>0</v>
-      </c>
-      <c r="O334" t="n">
-        <v>-1</v>
-      </c>
-      <c r="P334" t="n">
-        <v>-1</v>
-      </c>
-      <c r="Q334" t="n">
+      <c r="N334" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O334" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="P334" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="Q334" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="R334" t="n">
+      <c r="R334" s="0" t="n">
         <v>65</v>
       </c>
-      <c r="S334" t="n">
+      <c r="S334" s="0" t="n">
         <v>65</v>
       </c>
-      <c r="T334" t="n">
+      <c r="T334" s="0" t="n">
         <v>58</v>
       </c>
-      <c r="U334" t="n">
+      <c r="U334" s="0" t="n">
         <v>36</v>
       </c>
-      <c r="V334" t="n">
+      <c r="V334" s="0" t="n">
         <v>60</v>
       </c>
-      <c r="W334" t="n">
-        <v>0</v>
-      </c>
-      <c r="X334" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y334" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z334" t="n">
+      <c r="W334" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="X334" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y334" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z334" s="0" t="n">
         <v>45</v>
       </c>
-      <c r="AA334" t="n">
-        <v>10</v>
-      </c>
-      <c r="AB334" t="n">
+      <c r="AA334" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AB334" s="0" t="n">
         <v>15</v>
       </c>
-      <c r="AC334" t="n">
-        <v>10</v>
-      </c>
-      <c r="AD334" t="n">
+      <c r="AC334" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AD334" s="0" t="n">
         <v>25</v>
       </c>
-      <c r="AE334" t="n">
-        <v>10</v>
-      </c>
-      <c r="AF334" t="n">
-        <v>10</v>
-      </c>
-      <c r="AG334" t="n">
+      <c r="AE334" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AF334" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AG334" s="0" t="n">
         <v>42</v>
       </c>
-      <c r="AH334" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI334" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ334" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK334" t="n">
+      <c r="AH334" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI334" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ334" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK334" s="0" t="n">
         <v>50</v>
       </c>
-      <c r="AL334" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AM334" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN334" t="inlineStr">
+      <c r="AL334" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AM334" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN334" s="0" t="inlineStr">
         <is>
           <t>1,220</t>
         </is>
       </c>
-      <c r="AO334" t="n">
+      <c r="AO334" s="0" t="n">
         <v>-1</v>
       </c>
     </row>
     <row r="335">
-      <c r="A335" t="n">
+      <c r="A335" s="0" t="n">
         <v>330</v>
       </c>
-      <c r="B335" t="n">
+      <c r="B335" s="0" t="n">
         <v>71</v>
       </c>
-      <c r="C335" t="n">
+      <c r="C335" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="D335" t="inlineStr">
+      <c r="D335" s="0" t="inlineStr">
         <is>
           <t>西域三僧丙</t>
         </is>
       </c>
-      <c r="E335" t="inlineStr">
+      <c r="E335" s="0" t="inlineStr">
         <is>
           <t>西域三僧</t>
         </is>
       </c>
-      <c r="F335" t="n">
-        <v>0</v>
-      </c>
-      <c r="G335" t="n">
+      <c r="F335" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G335" s="0" t="n">
         <v>11</v>
       </c>
-      <c r="H335" t="n">
+      <c r="H335" s="0" t="n">
         <v>3050</v>
       </c>
-      <c r="I335" t="n">
+      <c r="I335" s="0" t="n">
         <v>190</v>
       </c>
-      <c r="J335" t="n">
+      <c r="J335" s="0" t="n">
         <v>190</v>
       </c>
-      <c r="K335" t="n">
-        <v>0</v>
-      </c>
-      <c r="L335" t="n">
-        <v>0</v>
-      </c>
-      <c r="M335" t="n">
+      <c r="K335" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="L335" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M335" s="0" t="n">
         <v>300</v>
       </c>
-      <c r="N335" t="n">
-        <v>0</v>
-      </c>
-      <c r="O335" t="n">
-        <v>-1</v>
-      </c>
-      <c r="P335" t="n">
-        <v>-1</v>
-      </c>
-      <c r="Q335" t="n">
+      <c r="N335" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O335" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="P335" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="Q335" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="R335" t="n">
+      <c r="R335" s="0" t="n">
         <v>65</v>
       </c>
-      <c r="S335" t="n">
+      <c r="S335" s="0" t="n">
         <v>65</v>
       </c>
-      <c r="T335" t="n">
+      <c r="T335" s="0" t="n">
         <v>58</v>
       </c>
-      <c r="U335" t="n">
+      <c r="U335" s="0" t="n">
         <v>36</v>
       </c>
-      <c r="V335" t="n">
+      <c r="V335" s="0" t="n">
         <v>60</v>
       </c>
-      <c r="W335" t="n">
-        <v>0</v>
-      </c>
-      <c r="X335" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y335" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z335" t="n">
+      <c r="W335" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="X335" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y335" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z335" s="0" t="n">
         <v>45</v>
       </c>
-      <c r="AA335" t="n">
-        <v>10</v>
-      </c>
-      <c r="AB335" t="n">
+      <c r="AA335" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AB335" s="0" t="n">
         <v>15</v>
       </c>
-      <c r="AC335" t="n">
-        <v>10</v>
-      </c>
-      <c r="AD335" t="n">
+      <c r="AC335" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AD335" s="0" t="n">
         <v>25</v>
       </c>
-      <c r="AE335" t="n">
-        <v>10</v>
-      </c>
-      <c r="AF335" t="n">
-        <v>10</v>
-      </c>
-      <c r="AG335" t="n">
+      <c r="AE335" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AF335" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AG335" s="0" t="n">
         <v>42</v>
       </c>
-      <c r="AH335" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI335" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ335" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK335" t="n">
+      <c r="AH335" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI335" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ335" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK335" s="0" t="n">
         <v>50</v>
       </c>
-      <c r="AL335" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AM335" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN335" t="inlineStr">
+      <c r="AL335" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AM335" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN335" s="0" t="inlineStr">
         <is>
           <t>1,220</t>
         </is>
       </c>
-      <c r="AO335" t="n">
+      <c r="AO335" s="0" t="n">
         <v>-1</v>
       </c>
     </row>
     <row r="336">
-      <c r="A336" t="n">
+      <c r="A336" s="0" t="n">
         <v>331</v>
       </c>
-      <c r="B336" t="n">
+      <c r="B336" s="0" t="n">
         <v>65</v>
       </c>
-      <c r="C336" t="n">
+      <c r="C336" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="D336" t="inlineStr">
+      <c r="D336" s="0" t="inlineStr">
         <is>
           <t>天鸣</t>
         </is>
       </c>
-      <c r="E336" t="inlineStr">
+      <c r="E336" s="0" t="inlineStr">
         <is>
           <t>少林高僧</t>
         </is>
       </c>
-      <c r="F336" t="n">
-        <v>0</v>
-      </c>
-      <c r="G336" t="n">
+      <c r="F336" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G336" s="0" t="n">
         <v>16</v>
       </c>
-      <c r="H336" t="n">
+      <c r="H336" s="0" t="n">
         <v>9250</v>
       </c>
-      <c r="I336" t="n">
+      <c r="I336" s="0" t="n">
         <v>250</v>
       </c>
-      <c r="J336" t="n">
+      <c r="J336" s="0" t="n">
         <v>250</v>
       </c>
-      <c r="K336" t="n">
-        <v>0</v>
-      </c>
-      <c r="L336" t="n">
-        <v>0</v>
-      </c>
-      <c r="M336" t="n">
+      <c r="K336" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="L336" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M336" s="0" t="n">
         <v>400</v>
       </c>
-      <c r="N336" t="n">
-        <v>0</v>
-      </c>
-      <c r="O336" t="n">
-        <v>-1</v>
-      </c>
-      <c r="P336" t="n">
-        <v>-1</v>
-      </c>
-      <c r="Q336" t="n">
+      <c r="N336" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O336" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="P336" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="Q336" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="R336" t="n">
+      <c r="R336" s="0" t="n">
         <v>85</v>
       </c>
-      <c r="S336" t="n">
+      <c r="S336" s="0" t="n">
         <v>85</v>
       </c>
-      <c r="T336" t="n">
+      <c r="T336" s="0" t="n">
         <v>70</v>
       </c>
-      <c r="U336" t="n">
+      <c r="U336" s="0" t="n">
         <v>45</v>
       </c>
-      <c r="V336" t="n">
+      <c r="V336" s="0" t="n">
         <v>76</v>
       </c>
-      <c r="W336" t="n">
-        <v>0</v>
-      </c>
-      <c r="X336" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y336" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z336" t="n">
+      <c r="W336" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="X336" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y336" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z336" s="0" t="n">
         <v>55</v>
       </c>
-      <c r="AA336" t="n">
-        <v>10</v>
-      </c>
-      <c r="AB336" t="n">
+      <c r="AA336" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AB336" s="0" t="n">
         <v>20</v>
       </c>
-      <c r="AC336" t="n">
-        <v>10</v>
-      </c>
-      <c r="AD336" t="n">
+      <c r="AC336" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AD336" s="0" t="n">
         <v>35</v>
       </c>
-      <c r="AE336" t="n">
-        <v>10</v>
-      </c>
-      <c r="AF336" t="n">
-        <v>10</v>
-      </c>
-      <c r="AG336" t="n">
+      <c r="AE336" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AF336" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AG336" s="0" t="n">
         <v>58</v>
       </c>
-      <c r="AH336" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI336" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ336" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK336" t="n">
+      <c r="AH336" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI336" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ336" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK336" s="0" t="n">
         <v>68</v>
       </c>
-      <c r="AL336" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AM336" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN336" t="inlineStr">
+      <c r="AL336" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AM336" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN336" s="0" t="inlineStr">
         <is>
           <t>1,320</t>
         </is>
       </c>
-      <c r="AO336" t="n">
+      <c r="AO336" s="0" t="n">
         <v>-1</v>
       </c>
     </row>
     <row r="337">
-      <c r="A337" t="n">
+      <c r="A337" s="0" t="n">
         <v>332</v>
       </c>
-      <c r="B337" t="n">
+      <c r="B337" s="0" t="n">
         <v>30</v>
       </c>
-      <c r="C337" t="n">
+      <c r="C337" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="D337" t="inlineStr">
+      <c r="D337" s="0" t="inlineStr">
         <is>
           <t>卓不凡</t>
         </is>
       </c>
-      <c r="E337" t="inlineStr">
+      <c r="E337" s="0" t="inlineStr">
         <is>
           <t>剑神</t>
         </is>
       </c>
-      <c r="F337" t="n">
-        <v>0</v>
-      </c>
-      <c r="G337" t="n">
+      <c r="F337" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G337" s="0" t="n">
         <v>22</v>
       </c>
-      <c r="H337" t="n">
+      <c r="H337" s="0" t="n">
         <v>21400</v>
       </c>
-      <c r="I337" t="n">
+      <c r="I337" s="0" t="n">
         <v>520</v>
       </c>
-      <c r="J337" t="n">
+      <c r="J337" s="0" t="n">
         <v>520</v>
       </c>
-      <c r="K337" t="n">
-        <v>0</v>
-      </c>
-      <c r="L337" t="n">
-        <v>0</v>
-      </c>
-      <c r="M337" t="n">
+      <c r="K337" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="L337" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M337" s="0" t="n">
         <v>650</v>
       </c>
-      <c r="N337" t="n">
-        <v>0</v>
-      </c>
-      <c r="O337" t="n">
-        <v>-1</v>
-      </c>
-      <c r="P337" t="n">
-        <v>-1</v>
-      </c>
-      <c r="Q337" t="n">
+      <c r="N337" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O337" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="P337" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="Q337" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="R337" t="n">
+      <c r="R337" s="0" t="n">
         <v>160</v>
       </c>
-      <c r="S337" t="n">
+      <c r="S337" s="0" t="n">
         <v>160</v>
       </c>
-      <c r="T337" t="n">
+      <c r="T337" s="0" t="n">
         <v>88</v>
       </c>
-      <c r="U337" t="n">
+      <c r="U337" s="0" t="n">
         <v>82</v>
       </c>
-      <c r="V337" t="n">
+      <c r="V337" s="0" t="n">
         <v>84</v>
       </c>
-      <c r="W337" t="n">
-        <v>0</v>
-      </c>
-      <c r="X337" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y337" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z337" t="n">
-        <v>10</v>
-      </c>
-      <c r="AA337" t="n">
-        <v>10</v>
-      </c>
-      <c r="AB337" t="n">
-        <v>10</v>
-      </c>
-      <c r="AC337" t="n">
-        <v>10</v>
-      </c>
-      <c r="AD337" t="n">
+      <c r="W337" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="X337" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y337" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z337" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AA337" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AB337" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AC337" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AD337" s="0" t="n">
         <v>92</v>
       </c>
-      <c r="AE337" t="n">
-        <v>10</v>
-      </c>
-      <c r="AF337" t="n">
+      <c r="AE337" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AF337" s="0" t="n">
         <v>88</v>
       </c>
-      <c r="AG337" t="n">
+      <c r="AG337" s="0" t="n">
         <v>65</v>
       </c>
-      <c r="AH337" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI337" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ337" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK337" t="n">
+      <c r="AH337" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI337" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ337" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK337" s="0" t="n">
         <v>75</v>
       </c>
-      <c r="AL337" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AM337" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN337" t="inlineStr">
+      <c r="AL337" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AM337" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN337" s="0" t="inlineStr">
         <is>
           <t>1,500</t>
         </is>
       </c>
-      <c r="AO337" t="n">
+      <c r="AO337" s="0" t="n">
         <v>-1</v>
       </c>
     </row>
     <row r="338">
-      <c r="A338" t="n">
+      <c r="A338" s="0" t="n">
         <v>333</v>
       </c>
-      <c r="B338" t="n">
+      <c r="B338" s="0" t="n">
         <v>19</v>
       </c>
-      <c r="C338" t="n">
+      <c r="C338" s="0" t="n">
         <v>8</v>
       </c>
-      <c r="D338" t="inlineStr">
+      <c r="D338" s="0" t="inlineStr">
         <is>
           <t>公孙止</t>
         </is>
       </c>
-      <c r="E338" t="inlineStr">
+      <c r="E338" s="0" t="inlineStr">
         <is>
           <t>绝情谷主</t>
         </is>
       </c>
-      <c r="F338" t="n">
-        <v>0</v>
-      </c>
-      <c r="G338" t="n">
+      <c r="F338" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G338" s="0" t="n">
         <v>24</v>
       </c>
-      <c r="H338" t="n">
+      <c r="H338" s="0" t="n">
         <v>28150</v>
       </c>
-      <c r="I338" t="n">
+      <c r="I338" s="0" t="n">
         <v>650</v>
       </c>
-      <c r="J338" t="n">
+      <c r="J338" s="0" t="n">
         <v>650</v>
       </c>
-      <c r="K338" t="n">
-        <v>0</v>
-      </c>
-      <c r="L338" t="n">
-        <v>0</v>
-      </c>
-      <c r="M338" t="n">
+      <c r="K338" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="L338" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M338" s="0" t="n">
         <v>720</v>
       </c>
-      <c r="N338" t="n">
-        <v>0</v>
-      </c>
-      <c r="O338" t="n">
-        <v>-1</v>
-      </c>
-      <c r="P338" t="n">
-        <v>-1</v>
-      </c>
-      <c r="Q338" t="n">
+      <c r="N338" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O338" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="P338" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="Q338" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="R338" t="n">
+      <c r="R338" s="0" t="n">
         <v>210</v>
       </c>
-      <c r="S338" t="n">
+      <c r="S338" s="0" t="n">
         <v>210</v>
       </c>
-      <c r="T338" t="n">
+      <c r="T338" s="0" t="n">
         <v>90</v>
       </c>
-      <c r="U338" t="n">
+      <c r="U338" s="0" t="n">
         <v>78</v>
       </c>
-      <c r="V338" t="n">
+      <c r="V338" s="0" t="n">
         <v>92</v>
       </c>
-      <c r="W338" t="n">
-        <v>0</v>
-      </c>
-      <c r="X338" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y338" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z338" t="n">
-        <v>10</v>
-      </c>
-      <c r="AA338" t="n">
-        <v>10</v>
-      </c>
-      <c r="AB338" t="n">
-        <v>10</v>
-      </c>
-      <c r="AC338" t="n">
-        <v>10</v>
-      </c>
-      <c r="AD338" t="n">
+      <c r="W338" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="X338" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y338" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z338" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AA338" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AB338" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AC338" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AD338" s="0" t="n">
         <v>86</v>
       </c>
-      <c r="AE338" t="n">
+      <c r="AE338" s="0" t="n">
         <v>80</v>
       </c>
-      <c r="AF338" t="n">
+      <c r="AF338" s="0" t="n">
         <v>60</v>
       </c>
-      <c r="AG338" t="n">
+      <c r="AG338" s="0" t="n">
         <v>70</v>
       </c>
-      <c r="AH338" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI338" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ338" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK338" t="n">
+      <c r="AH338" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI338" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ338" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK338" s="0" t="n">
         <v>70</v>
       </c>
-      <c r="AL338" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AM338" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN338" t="inlineStr">
+      <c r="AL338" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AM338" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN338" s="0" t="inlineStr">
         <is>
           <t>1,600</t>
         </is>
       </c>
-      <c r="AO338" t="n">
+      <c r="AO338" s="0" t="n">
         <v>-1</v>
       </c>
     </row>
     <row r="339">
-      <c r="A339" t="n">
+      <c r="A339" s="0" t="n">
         <v>334</v>
       </c>
-      <c r="B339" t="n">
+      <c r="B339" s="0" t="n">
         <v>63</v>
       </c>
-      <c r="C339" t="n">
+      <c r="C339" s="0" t="n">
         <v>9</v>
       </c>
-      <c r="D339" t="inlineStr">
+      <c r="D339" s="0" t="inlineStr">
         <is>
           <t>九天玄女</t>
         </is>
       </c>
-      <c r="E339" t="inlineStr">
+      <c r="E339" s="0" t="inlineStr">
         <is>
           <t>天上玄女</t>
         </is>
       </c>
-      <c r="F339" t="n">
+      <c r="F339" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="G339" t="n">
+      <c r="G339" s="0" t="n">
         <v>35</v>
       </c>
-      <c r="H339" t="n">
+      <c r="H339" s="0" t="n">
         <v>-9036</v>
       </c>
-      <c r="I339" t="n">
+      <c r="I339" s="0" t="n">
         <v>900</v>
       </c>
-      <c r="J339" t="n">
+      <c r="J339" s="0" t="n">
         <v>900</v>
       </c>
-      <c r="K339" t="n">
-        <v>0</v>
-      </c>
-      <c r="L339" t="n">
-        <v>0</v>
-      </c>
-      <c r="M339" t="n">
+      <c r="K339" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="L339" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M339" s="0" t="n">
         <v>999</v>
       </c>
-      <c r="N339" t="n">
-        <v>0</v>
-      </c>
-      <c r="O339" t="n">
-        <v>-1</v>
-      </c>
-      <c r="P339" t="n">
-        <v>-1</v>
-      </c>
-      <c r="Q339" t="n">
+      <c r="N339" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O339" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="P339" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="Q339" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="R339" t="n">
+      <c r="R339" s="0" t="n">
         <v>999</v>
       </c>
-      <c r="S339" t="n">
+      <c r="S339" s="0" t="n">
         <v>999</v>
       </c>
-      <c r="T339" t="n">
+      <c r="T339" s="0" t="n">
         <v>99</v>
       </c>
-      <c r="U339" t="n">
+      <c r="U339" s="0" t="n">
         <v>99</v>
       </c>
-      <c r="V339" t="n">
+      <c r="V339" s="0" t="n">
         <v>99</v>
       </c>
-      <c r="W339" t="n">
-        <v>0</v>
-      </c>
-      <c r="X339" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y339" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z339" t="n">
-        <v>10</v>
-      </c>
-      <c r="AA339" t="n">
-        <v>10</v>
-      </c>
-      <c r="AB339" t="n">
-        <v>10</v>
-      </c>
-      <c r="AC339" t="n">
-        <v>10</v>
-      </c>
-      <c r="AD339" t="n">
+      <c r="W339" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="X339" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y339" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z339" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AA339" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AB339" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AC339" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AD339" s="0" t="n">
         <v>99</v>
       </c>
-      <c r="AE339" t="n">
-        <v>10</v>
-      </c>
-      <c r="AF339" t="n">
+      <c r="AE339" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="AF339" s="0" t="n">
         <v>99</v>
       </c>
-      <c r="AG339" t="n">
+      <c r="AG339" s="0" t="n">
         <v>90</v>
       </c>
-      <c r="AH339" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI339" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ339" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK339" t="n">
+      <c r="AH339" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI339" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ339" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK339" s="0" t="n">
         <v>99</v>
       </c>
-      <c r="AL339" t="n">
-        <v>-1</v>
-      </c>
-      <c r="AM339" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN339" t="inlineStr">
+      <c r="AL339" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AM339" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN339" s="0" t="inlineStr">
         <is>
           <t>61,900</t>
         </is>
       </c>
-      <c r="AO339" t="n">
+      <c r="AO339" s="0" t="n">
         <v>-1</v>
       </c>
     </row>

</xml_diff>